<commit_message>
Rename employment templates to 雇用契約書兼労働条件通知書 across site content, navigation, and spreadsheet downloads.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/public/downloads/employment-contract-sabikan.xlsx
+++ b/docs/public/downloads/employment-contract-sabikan.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="労働条件通知書" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="雇用契約書兼労働条件通知書" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
-    <t>労 働 条 件 通 知 書</t>
+    <t>雇用契約書兼労働条件通知書</t>
   </si>
   <si>
     <t>氏名　〇〇（サビ管）　殿</t>
@@ -29,8 +29,8 @@
   </si>
   <si>
     <t xml:space="preserve">契約の更新の有無
-・更新する場合がある
-・契約の更新はしない
+☐ 更新する場合がある
+☐ 契約の更新はしない
 契約の更新は次により判断する
 ・契約期間満了時の業務量
 ・勤務成績、勤務態度
@@ -42,7 +42,9 @@
     <t>雇用形態</t>
   </si>
   <si>
-    <t>有期契約社員（※開設企業の雇用形態に合わせて修正）</t>
+    <t xml:space="preserve">☐ 正社員（期間の定めなし）
+☐ 有期契約社員
+☐ パート・アルバイト</t>
   </si>
   <si>
     <t>就業の場所</t>
@@ -73,9 +75,9 @@
   </si>
   <si>
     <t xml:space="preserve">1. 所定時間外労働の有無
+   ☐ 有　　☐ 無
 2. 休日労働の有無
-・ 有
-・ 有</t>
+   ☐ 有　　☐ 無</t>
   </si>
   <si>
     <t>休 日</t>
@@ -106,17 +108,17 @@
 ・ 当月　末
 ・ 翌月　20日
 ・ 所得税、雇用保険、健康保険、厚生年金
-・ 年次昇給有</t>
+・ 昇給　☐ 年次昇給有　　☐ なし</t>
   </si>
   <si>
     <t>退 職 に 関 す る 事 項</t>
   </si>
   <si>
     <t xml:space="preserve">1. 定年制
+   ☐ 有　　☐ 無
 2. 自己都合退職の手続
+・ 30日以上前までに届出が必要
 3. 解雇の事由及び手続
-・ 無
-・ 30日以上前までに届出が必要
 ・ 詳細は、就業規則による</t>
   </si>
   <si>
@@ -124,9 +126,9 @@
   </si>
   <si>
     <t xml:space="preserve">・社会保険の加入
+   ☐ 有　　☐ 無
 ・雇用保険の適用
-・ 有
-・ 有</t>
+   ☐ 有　　☐ 無</t>
   </si>
   <si>
     <t xml:space="preserve">解雇、退職、懲戒、
@@ -179,7 +181,7 @@
     <font>
       <b/>
       <color rgb="FF1E3A5F"/>
-      <sz val="16"/>
+      <sz val="14"/>
       <name val="Yu Gothic"/>
     </font>
     <font>
@@ -625,7 +627,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -778,13 +780,9 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>9</v>
-      </c>
+    <row r="15" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
@@ -792,7 +790,7 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -803,8 +801,12 @@
       <c r="H16" s="4"/>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
+      <c r="A17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
@@ -822,13 +824,9 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>11</v>
-      </c>
+    <row r="19" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
@@ -836,33 +834,37 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+    <row r="20" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
@@ -881,12 +883,8 @@
       <c r="H23" s="5"/>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A24" s="3"/>
+      <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
@@ -905,8 +903,12 @@
       <c r="H25" s="5"/>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="5"/>
+      <c r="A26" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
@@ -924,13 +926,9 @@
       <c r="G27" s="5"/>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>17</v>
-      </c>
+    <row r="28" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
@@ -938,13 +936,9 @@
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
     </row>
-    <row r="29" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>19</v>
-      </c>
+    <row r="29" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="3"/>
+      <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
@@ -953,8 +947,12 @@
       <c r="H29" s="5"/>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="5"/>
+      <c r="A30" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
@@ -962,33 +960,37 @@
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
     </row>
-    <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B33" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-    </row>
-    <row r="32" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
@@ -1097,32 +1099,32 @@
       <c r="H43" s="4"/>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
+      <c r="A44" s="3"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="3"/>
-      <c r="B46" s="5"/>
+      <c r="A46" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
       <c r="E46" s="5"/>
@@ -1160,13 +1162,9 @@
       <c r="G49" s="5"/>
       <c r="H49" s="5"/>
     </row>
-    <row r="50" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>25</v>
-      </c>
+    <row r="50" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="3"/>
+      <c r="B50" s="5"/>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
@@ -1174,7 +1172,7 @@
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
     </row>
-    <row r="51" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -1185,8 +1183,12 @@
       <c r="H51" s="5"/>
     </row>
     <row r="52" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
-      <c r="B52" s="5"/>
+      <c r="A52" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
@@ -1204,13 +1206,9 @@
       <c r="G53" s="5"/>
       <c r="H53" s="5"/>
     </row>
-    <row r="54" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>27</v>
-      </c>
+    <row r="54" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="3"/>
+      <c r="B54" s="5"/>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
@@ -1218,13 +1216,9 @@
       <c r="G54" s="5"/>
       <c r="H54" s="5"/>
     </row>
-    <row r="55" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>29</v>
-      </c>
+    <row r="55" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="3"/>
+      <c r="B55" s="5"/>
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
@@ -1232,9 +1226,13 @@
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
     </row>
-    <row r="56" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" s="3"/>
-      <c r="B56" s="5"/>
+    <row r="56" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
@@ -1242,45 +1240,45 @@
       <c r="G56" s="5"/>
       <c r="H56" s="5"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="6" t="s">
+    <row r="57" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+    </row>
+    <row r="58" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="3"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="6"/>
-      <c r="F58" s="6"/>
-      <c r="G58" s="6"/>
-      <c r="H58" s="6"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-      <c r="D60" s="7"/>
-      <c r="E60" s="7"/>
-      <c r="F60" s="7"/>
-      <c r="G60" s="7"/>
-      <c r="H60" s="7"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B61" s="7"/>
-      <c r="C61" s="7"/>
-      <c r="D61" s="7"/>
-      <c r="E61" s="7"/>
-      <c r="F61" s="7"/>
-      <c r="G61" s="7"/>
-      <c r="H61" s="7"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="6"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7"/>
@@ -1290,76 +1288,101 @@
       <c r="G62" s="7"/>
       <c r="H62" s="7"/>
     </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+    </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B64" s="8"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="9" t="s">
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="9" t="s">
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="9"/>
+      <c r="G67" s="9"/>
+      <c r="H67" s="9"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
-      <c r="H66" s="9"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="9"/>
+      <c r="G68" s="9"/>
+      <c r="H68" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="33">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B5:H13"/>
     <mergeCell ref="A5:A13"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B15:H18"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B20:H23"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="B24:H27"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="B28:H28"/>
-    <mergeCell ref="B29:H30"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B31:H43"/>
-    <mergeCell ref="A31:A43"/>
-    <mergeCell ref="B44:H49"/>
-    <mergeCell ref="A44:A49"/>
-    <mergeCell ref="B50:H53"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="B54:H54"/>
-    <mergeCell ref="B55:H56"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="B14:H16"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B17:H20"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B22:H25"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B26:H29"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="B31:H32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B33:H45"/>
+    <mergeCell ref="A33:A45"/>
+    <mergeCell ref="B46:H51"/>
+    <mergeCell ref="A46:A51"/>
+    <mergeCell ref="B52:H55"/>
+    <mergeCell ref="A52:A55"/>
+    <mergeCell ref="B56:H56"/>
+    <mergeCell ref="B57:H58"/>
+    <mergeCell ref="A57:A58"/>
     <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A61:H61"/>
     <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A63:H63"/>
     <mergeCell ref="A64:H64"/>
-    <mergeCell ref="A65:H65"/>
     <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A68:H68"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Fix clipped label text in employment contract spreadsheets and web templates.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/public/downloads/employment-contract-sabikan.xlsx
+++ b/docs/public/downloads/employment-contract-sabikan.xlsx
@@ -132,7 +132,8 @@
   </si>
   <si>
     <t xml:space="preserve">解雇、退職、懲戒、
-服務規律、契約解除、その他</t>
+服務規律、契約解除、
+その他</t>
   </si>
   <si>
     <t>・甲は雇用において、乙の執務態度、能力、成績、勤怠などについて不適格と認める場合は解雇する。また試用期間終了時において乙の執務態度、能力、成績、勤怠などについて不適格と認められた場合は試用期間満了とし、契約を解除する</t>
@@ -142,7 +143,7 @@
   </si>
   <si>
     <t xml:space="preserve">・この雇用契約書に定めのない事項については労働基準法及び就業規則の定める所による
-本契約書は甲乙1部ずつ作成し、各々で保管する。</t>
+・本契約書は甲乙1部ずつ作成し、各々で保管する。</t>
   </si>
   <si>
     <t>令和　　　年　　　月　　　日</t>
@@ -265,7 +266,7 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -627,7 +628,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -946,7 +947,7 @@
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
     </row>
-    <row r="30" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>16</v>
       </c>
@@ -960,7 +961,7 @@
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
     </row>
-    <row r="31" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>18</v>
       </c>
@@ -974,7 +975,7 @@
       <c r="G31" s="5"/>
       <c r="H31" s="5"/>
     </row>
-    <row r="32" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1182,7 +1183,7 @@
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
     </row>
-    <row r="52" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>24</v>
       </c>
@@ -1196,7 +1197,7 @@
       <c r="G52" s="5"/>
       <c r="H52" s="5"/>
     </row>
-    <row r="53" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
@@ -1206,7 +1207,7 @@
       <c r="G53" s="5"/>
       <c r="H53" s="5"/>
     </row>
-    <row r="54" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -1216,7 +1217,7 @@
       <c r="G54" s="5"/>
       <c r="H54" s="5"/>
     </row>
-    <row r="55" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -1226,7 +1227,7 @@
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
     </row>
-    <row r="56" ht="36" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>26</v>
       </c>
@@ -1240,13 +1241,9 @@
       <c r="G56" s="5"/>
       <c r="H56" s="5"/>
     </row>
-    <row r="57" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>29</v>
-      </c>
+    <row r="57" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="3"/>
+      <c r="B57" s="5"/>
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
@@ -1254,7 +1251,7 @@
       <c r="G57" s="5"/>
       <c r="H57" s="5"/>
     </row>
-    <row r="58" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -1264,92 +1261,136 @@
       <c r="G58" s="5"/>
       <c r="H58" s="5"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="6" t="s">
+    <row r="59" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="3"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+    </row>
+    <row r="60" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="3"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+    </row>
+    <row r="62" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="3"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="6"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
-      <c r="F60" s="6"/>
-      <c r="G60" s="6"/>
-      <c r="H60" s="6"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="7" t="s">
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="6"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7"/>
-      <c r="F62" s="7"/>
-      <c r="G62" s="7"/>
-      <c r="H62" s="7"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A63" s="7" t="s">
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7"/>
+      <c r="G66" s="7"/>
+      <c r="H66" s="7"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B63" s="7"/>
-      <c r="C63" s="7"/>
-      <c r="D63" s="7"/>
-      <c r="E63" s="7"/>
-      <c r="F63" s="7"/>
-      <c r="G63" s="7"/>
-      <c r="H63" s="7"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="7" t="s">
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B64" s="7"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-      <c r="H64" s="7"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="8" t="s">
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="7"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="7"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B66" s="8"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="8"/>
-      <c r="E66" s="8"/>
-      <c r="F66" s="8"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="8"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" s="9" t="s">
+      <c r="B70" s="8"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="8"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A68" s="9" t="s">
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9"/>
+      <c r="G71" s="9"/>
+      <c r="H71" s="9"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
-      <c r="H68" s="9"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9"/>
+      <c r="F72" s="9"/>
+      <c r="G72" s="9"/>
+      <c r="H72" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B4:H4"/>
@@ -1373,16 +1414,17 @@
     <mergeCell ref="A46:A51"/>
     <mergeCell ref="B52:H55"/>
     <mergeCell ref="A52:A55"/>
-    <mergeCell ref="B56:H56"/>
-    <mergeCell ref="B57:H58"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A62:H62"/>
-    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="B56:H60"/>
+    <mergeCell ref="A56:A60"/>
+    <mergeCell ref="B61:H62"/>
+    <mergeCell ref="A61:A62"/>
     <mergeCell ref="A64:H64"/>
     <mergeCell ref="A66:H66"/>
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A70:H70"/>
+    <mergeCell ref="A71:H71"/>
+    <mergeCell ref="A72:H72"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Tighten employment contract spreadsheet row heights to reduce excess whitespace.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/public/downloads/employment-contract-sabikan.xlsx
+++ b/docs/public/downloads/employment-contract-sabikan.xlsx
@@ -51,8 +51,7 @@
   </si>
   <si>
     <t xml:space="preserve">〇〇県〇〇市〇〇1-2-3　〇〇就労継続支援B型事業所
-（複数事業所がある場合は行を追加）
-</t>
+（複数事業所がある場合は行を追加）</t>
   </si>
   <si>
     <t>従事する業務の内容</t>
@@ -628,7 +627,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -825,9 +824,13 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4"/>
+    <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
@@ -835,37 +838,33 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
+    <row r="20" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>13</v>
-      </c>
+      <c r="A22" s="3"/>
+      <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
@@ -884,8 +883,12 @@
       <c r="H23" s="5"/>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="B24" s="5"/>
+      <c r="A24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
@@ -904,12 +907,8 @@
       <c r="H25" s="5"/>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="A26" s="3"/>
+      <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
@@ -928,8 +927,12 @@
       <c r="H27" s="5"/>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="B28" s="5"/>
+      <c r="A28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
@@ -938,8 +941,12 @@
       <c r="H28" s="5"/>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="5"/>
+      <c r="A29" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
@@ -948,12 +955,8 @@
       <c r="H29" s="5"/>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="A30" s="3"/>
+      <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
@@ -963,35 +966,31 @@
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
+        <v>20</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
     </row>
     <row r="32" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>21</v>
-      </c>
+      <c r="A33" s="3"/>
+      <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
@@ -1100,32 +1099,32 @@
       <c r="H43" s="4"/>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="3"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
+      <c r="A44" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>23</v>
-      </c>
+      <c r="A46" s="3"/>
+      <c r="B46" s="5"/>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
       <c r="E46" s="5"/>
@@ -1164,8 +1163,12 @@
       <c r="H49" s="5"/>
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="3"/>
-      <c r="B50" s="5"/>
+      <c r="A50" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
@@ -1184,12 +1187,8 @@
       <c r="H51" s="5"/>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="A52" s="3"/>
+      <c r="B52" s="5"/>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
@@ -1208,8 +1207,12 @@
       <c r="H53" s="5"/>
     </row>
     <row r="54" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-      <c r="B54" s="5"/>
+      <c r="A54" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
@@ -1227,13 +1230,9 @@
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
     </row>
-    <row r="56" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>27</v>
-      </c>
+    <row r="56" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="3"/>
+      <c r="B56" s="5"/>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
@@ -1241,9 +1240,13 @@
       <c r="G56" s="5"/>
       <c r="H56" s="5"/>
     </row>
-    <row r="57" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="3"/>
-      <c r="B57" s="5"/>
+    <row r="57" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
@@ -1251,7 +1254,7 @@
       <c r="G57" s="5"/>
       <c r="H57" s="5"/>
     </row>
-    <row r="58" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
@@ -1261,133 +1264,89 @@
       <c r="G58" s="5"/>
       <c r="H58" s="5"/>
     </row>
-    <row r="59" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="3"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-    </row>
-    <row r="60" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="3"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
-      <c r="H60" s="5"/>
-    </row>
-    <row r="61" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-    </row>
-    <row r="62" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="3"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="6"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="6"/>
-      <c r="F64" s="6"/>
-      <c r="G64" s="6"/>
-      <c r="H64" s="6"/>
+      <c r="A64" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
-      <c r="F66" s="7"/>
-      <c r="G66" s="7"/>
-      <c r="H66" s="7"/>
+      <c r="A66" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B67" s="7"/>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7"/>
-      <c r="E67" s="7"/>
-      <c r="F67" s="7"/>
-      <c r="G67" s="7"/>
-      <c r="H67" s="7"/>
+      <c r="A67" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9"/>
+      <c r="F67" s="9"/>
+      <c r="G67" s="9"/>
+      <c r="H67" s="9"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A68" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B68" s="7"/>
-      <c r="C68" s="7"/>
-      <c r="D68" s="7"/>
-      <c r="E68" s="7"/>
-      <c r="F68" s="7"/>
-      <c r="G68" s="7"/>
-      <c r="H68" s="7"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B70" s="8"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="8"/>
-      <c r="E70" s="8"/>
-      <c r="F70" s="8"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="8"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A71" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
-      <c r="F71" s="9"/>
-      <c r="G71" s="9"/>
-      <c r="H71" s="9"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" s="9" t="s">
+      <c r="A68" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
-      <c r="G72" s="9"/>
-      <c r="H72" s="9"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="9"/>
+      <c r="G68" s="9"/>
+      <c r="H68" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="34">
@@ -1398,33 +1357,33 @@
     <mergeCell ref="A5:A13"/>
     <mergeCell ref="B14:H16"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B17:H20"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B22:H25"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="B26:H29"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B31:H32"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B33:H45"/>
-    <mergeCell ref="A33:A45"/>
-    <mergeCell ref="B46:H51"/>
-    <mergeCell ref="A46:A51"/>
-    <mergeCell ref="B52:H55"/>
-    <mergeCell ref="A52:A55"/>
-    <mergeCell ref="B56:H60"/>
-    <mergeCell ref="A56:A60"/>
-    <mergeCell ref="B61:H62"/>
-    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="B17:H18"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B20:H23"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="B24:H27"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B29:H30"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B31:H43"/>
+    <mergeCell ref="A31:A43"/>
+    <mergeCell ref="B44:H49"/>
+    <mergeCell ref="A44:A49"/>
+    <mergeCell ref="B50:H53"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="B54:H56"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B57:H58"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A63:H63"/>
     <mergeCell ref="A64:H64"/>
     <mergeCell ref="A66:H66"/>
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A70:H70"/>
-    <mergeCell ref="A71:H71"/>
-    <mergeCell ref="A72:H72"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>